<commit_message>
refactor(output): update audit prompt instructions and rubric
Update the moorage audit prompt files to reflect new instructions regarding
post-adoption length amendments, priority tier classification, and
reconciliation procedures. Also update the rubric summary spreadsheet to
align with these changes.
</commit_message>
<xml_diff>
--- a/output/rubric_summary.xlsx
+++ b/output/rubric_summary.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">Model</t>
   </si>
@@ -31,36 +31,24 @@
     <t xml:space="preserve">Rsponse 1</t>
   </si>
   <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAIL - need ≥8 fails (have 6)</t>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">53%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS - meets ≥50% fail threshold</t>
   </si>
   <si>
     <t xml:space="preserve">Response 2</t>
   </si>
   <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">53%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">46%</t>
-  </si>
-  <si>
     <t xml:space="preserve"/>
   </si>
   <si>
@@ -79,9 +67,6 @@
     <t xml:space="preserve">80%</t>
   </si>
   <si>
-    <t xml:space="preserve">PASS - meets ≥80% fail threshold (weakest)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Response 4</t>
   </si>
   <si>
@@ -94,7 +79,7 @@
     <t xml:space="preserve">33%</t>
   </si>
   <si>
-    <t xml:space="preserve">66%</t>
+    <t xml:space="preserve">67%</t>
   </si>
   <si>
     <t xml:space="preserve">Response 5</t>
@@ -109,7 +94,7 @@
     <t xml:space="preserve">Response 8</t>
   </si>
   <si>
-    <t xml:space="preserve">FAIL - need ≥12 fails (have 5)</t>
+    <t xml:space="preserve">PASS - meets ≥80% fail threshold</t>
   </si>
 </sst>
 </file>
@@ -162,139 +147,139 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
         <v>28</v>
-      </c>
-      <c r="E9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(output): define explicit criteria for exception priority tiers
Update the audit prompt instructions to replace subjective priority
classification with specific, predefined criteria for Priority 1, 2,
and 3 tiers. This ensures consistent classification of skips and
post-adoption amendments.
</commit_message>
<xml_diff>
--- a/output/rubric_summary.xlsx
+++ b/output/rubric_summary.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">Model</t>
   </si>
@@ -43,12 +43,24 @@
     <t xml:space="preserve">53%</t>
   </si>
   <si>
-    <t xml:space="preserve">PASS - meets ≥50% fail threshold</t>
+    <t xml:space="preserve">PASS - fails ≥50% of critical elements</t>
   </si>
   <si>
     <t xml:space="preserve">Response 2</t>
   </si>
   <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60%</t>
+  </si>
+  <si>
     <t xml:space="preserve"/>
   </si>
   <si>
@@ -94,7 +106,7 @@
     <t xml:space="preserve">Response 8</t>
   </si>
   <si>
-    <t xml:space="preserve">PASS - meets ≥80% fail threshold</t>
+    <t xml:space="preserve">PASS - fails ≥80% of critical elements</t>
   </si>
 </sst>
 </file>
@@ -147,139 +159,139 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>